<commit_message>
Switch costs spreadsheet currency to US dollars
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lsb4HXzKkpncstus3MhoPF
</commit_message>
<xml_diff>
--- a/new-company/new-company-costs.xlsx
+++ b/new-company/new-company-costs.xlsx
@@ -22,7 +22,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="&quot;R$&quot; #,##0.00;(&quot;R$&quot; #,##0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -583,7 +583,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Unit cost (R$)</t>
+          <t>Unit cost (US$)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Total (R$)</t>
+          <t>Total (US$)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -8762,37 +8762,37 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>One-time actual (R$)</t>
+          <t>One-time actual (US$)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>One-time possible (R$)</t>
+          <t>One-time possible (US$)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Monthly actual (R$)</t>
+          <t>Monthly actual (US$)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Monthly possible (R$)</t>
+          <t>Monthly possible (US$)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Total actual (horizon) (R$)</t>
+          <t>Total actual (horizon) (US$)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Total possible (horizon) (R$)</t>
+          <t>Total possible (horizon) (US$)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Grand total (horizon) (R$)</t>
+          <t>Grand total (horizon) (US$)</t>
         </is>
       </c>
     </row>
@@ -9160,37 +9160,37 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>One-time actual (R$)</t>
+          <t>One-time actual (US$)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>One-time possible (R$)</t>
+          <t>One-time possible (US$)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Monthly actual (R$)</t>
+          <t>Monthly actual (US$)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Monthly possible (R$)</t>
+          <t>Monthly possible (US$)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Total actual (horizon) (R$)</t>
+          <t>Total actual (horizon) (US$)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Total possible (horizon) (R$)</t>
+          <t>Total possible (horizon) (US$)</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Grand total (horizon) (R$)</t>
+          <t>Grand total (horizon) (US$)</t>
         </is>
       </c>
     </row>

</xml_diff>